<commit_message>
Import real color scale rules from XLSX (<colorScale>/<cfvo>)
<cfRule type="colorScale"> doesn't use dxfId like cellIs/duplicateValues
-- its colors and thresholds are inline in a <colorScale> child element
(<cfvo type="min|max|percentile|percent|num" val="..."/> paired
positionally with <color rgb="..."/>). ParseSheet now collects these
into CondFormatRule::csCfvos/csColors, and ApplyConditionalFormatting
converts a rule with 2+ matching cfvo/color pairs into a real
eCondColorScale engine rule instead of silently discarding it.

Extends tests/sample_condformat.xlsx with a third rule (colorScale on
C1:C10, min/percentile-50/max) and updates test_xlsx_translator.cpp's
manual ASCD byte-parser to verify all three control points and their
colors survive the import, not just skip past them.
</commit_message>
<xml_diff>
--- a/translators/xlsx/tests/sample_condformat.xlsx
+++ b/translators/xlsx/tests/sample_condformat.xlsx
@@ -105,5 +105,17 @@
   <conditionalFormatting sqref="B1:B3">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C1:C10">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
</xml_diff>